<commit_message>
Ministries (M2): real ministries everywhere
db/023 makes the member directory list each member's real ministries,
so the directory, Dashboard and Reports use them; db/024 fixes members
not being able to see their own ministries. The Members page shows real
ministries and no longer sets one (the Pastor or a ministry's head
assigns), the Excel import and template drop the Ministry column, the
Events form lists the branch's real ministries, Reports counts members
in every ministry they're in, and members get a My ministries page and
a real count on their home page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/faithsync-members-template.xlsx
+++ b/public/templates/faithsync-members-template.xlsx
@@ -23,9 +23,6 @@
     <t>Role</t>
   </si>
   <si>
-    <t>Ministry</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
@@ -41,9 +38,6 @@
     <t>member</t>
   </si>
   <si>
-    <t>Program &amp; Music Ministry</t>
-  </si>
-  <si>
     <t>09171234567</t>
   </si>
   <si>
@@ -62,9 +56,6 @@
     <t>leader</t>
   </si>
   <si>
-    <t>Mission &amp; Evangelism</t>
-  </si>
-  <si>
     <t>busy</t>
   </si>
   <si>
@@ -74,9 +65,6 @@
     <t>volunteer</t>
   </si>
   <si>
-    <t>Training &amp; Life Ministry</t>
-  </si>
-  <si>
     <t>inactive</t>
   </si>
   <si>
@@ -86,13 +74,7 @@
     <t>pastor</t>
   </si>
   <si>
-    <t>Building &amp; Equipment</t>
-  </si>
-  <si>
-    <t>Use these exact words for Role, Ministry and Status.</t>
-  </si>
-  <si>
-    <t>Finance Ministry</t>
+    <t>Ministries are added later on the Ministries page.</t>
   </si>
 </sst>
 </file>
@@ -141,10 +123,9 @@
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -163,28 +144,22 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -195,9 +170,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="55" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -205,71 +179,51 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="s">
-        <v>25</v>
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove Busy status; Leaders see own ministries; ministry tiles; Next Schedule on top; simpler event cards
</commit_message>
<xml_diff>
--- a/public/templates/faithsync-members-template.xlsx
+++ b/public/templates/faithsync-members-template.xlsx
@@ -214,7 +214,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
@@ -224,9 +224,6 @@
       <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
       <c r="C4" t="s">
         <v>17</v>
       </c>

</xml_diff>